<commit_message>
Fix OpenAI Ads XLSX: rename sheet to 'campaigns'
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K23AdRzfbK9DAxfNeDXX3m
</commit_message>
<xml_diff>
--- a/output/openai-ads-kampanie.xlsx
+++ b/output/openai-ads-kampanie.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="OpenAI Ads Kampanie" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="campaigns" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Uwagi" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,9 +30,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -99,7 +96,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -735,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -785,7 +782,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>ID lokalizacji (opcjonalne - dla Warszawa)</t>
+          <t>ID lokalizacji (opcjonalne)</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -802,29 +799,12 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Zostaw puste = wszystkie platformy</t>
+          <t>Zostaw puste = wszystkie</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
           <t>lub wpisz: chatgpt / browsing</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>budget_max</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Kwota dzienna w PLN</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Możesz zmienić przed uruchomieniem</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add adgroups sheet to OpenAI Ads XLSX
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K23AdRzfbK9DAxfNeDXX3m
</commit_message>
<xml_diff>
--- a/output/openai-ads-kampanie.xlsx
+++ b/output/openai-ads-kampanie.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="campaigns" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Uwagi" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="adgroups" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Uwagi" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,10 +31,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="5">
@@ -85,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -96,7 +93,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -732,79 +728,286 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>adgroup_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>adgroup_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>campaign_name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Zaręczyny Warszawa</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Pierścionki Warszawa</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr"/>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Pierścionki na zamówienie</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Pierścionki Warszawa</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Diamenty certyfikowane</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Pierścionki Ogólne</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Pierścionek zaręczynowy</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Pierścionki Ogólne</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Skup diamentów Warszawa</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Wycena i skup diamentów</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Wycena brylantów</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Wycena i skup diamentów</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Certyfikat GIA IGI</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Ekspertyzy i gemmologia</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Gemmolog Warszawa</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Ekspertyzy i gemmologia</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Forum Jubiler marka</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Forum Jubiler brand</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Pole</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Co wpisać</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Gdzie znaleźć</t>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Opis</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>campaign_id / adgroup_id</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Zostaw puste — OpenAI Ads uzupełni automatycznie po imporcie</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>conversion_event_setting_ids</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>ID zdarzenia konwersji z panelu OpenAI</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>OpenAI Ads → Conversions → skopiuj ID</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Skopiuj ID z panelu: OpenAI Ads → Conversions</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>location_ids</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>ID lokalizacji (opcjonalne)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>OpenAI Ads → kampania → Location targeting</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Opcjonalne — ID lokalizacji dla targetowania geograficznego</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>platforms</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Zostaw puste = wszystkie</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>lub wpisz: chatgpt / browsing</t>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Puste = wszystkie; lub: chatgpt / browsing</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>ACTIVE lub PAUSED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ads sheet to OpenAI Ads XLSX (campaigns + adgroups + ads)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K23AdRzfbK9DAxfNeDXX3m
</commit_message>
<xml_diff>
--- a/output/openai-ads-kampanie.xlsx
+++ b/output/openai-ads-kampanie.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="campaigns" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="adgroups" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Uwagi" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ads" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -82,18 +82,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -932,82 +931,349 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Pole</t>
+          <t>ad_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Opis</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>campaign_id / adgroup_id</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Zostaw puste — OpenAI Ads uzupełni automatycznie po imporcie</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>conversion_event_setting_ids</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Skopiuj ID z panelu: OpenAI Ads → Conversions</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>location_ids</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Opcjonalne — ID lokalizacji dla targetowania geograficznego</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>platforms</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Puste = wszystkie; lub: chatgpt / browsing</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+          <t>ad_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>adgroup_name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>headline</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>final_url</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>ACTIVE lub PAUSED</t>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Zaręczyny Warszawa – Pierścionki</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Zaręczyny Warszawa</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Pierścionki zaręczynowe Warszawa</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Złoto 18k, platyna, brylant z certyfikatem GIA. Projekt 3D gratis. Forum Jubiler – Chłodna 22.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://forumjubiler.pl/pierscionki-zareczynowe</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="3" t="inlineStr"/>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Pierścionki na zamówienie – 1</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Pierścionki na zamówienie</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Pierścionek na zamówienie Warszawa</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Własny projekt w 3D, złoto 18k lub platyna. 3 miesiące na zmianę rozmiaru. Umów wizytę.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>https://forumjubiler.pl/pierscionki-zareczynowe</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Diamenty certyfikowane – 1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Diamenty certyfikowane</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Diament z certyfikatem GIA lub IGI</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Szeroki wybór brylantów certyfikowanych. Bezpłatna wycena kamienia. Forum Jubiler od 1992 r.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>https://forumjubiler.pl/diamenty</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Pierścionek zaręczynowy – 1</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Pierścionek zaręczynowy</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Pierścionek zaręczynowy z brylantem</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Certyfikowany diament, złoto 18k lub platyna. Projekt 3D + korekta rozmiaru gratis.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>https://forumjubiler.pl/pierscionki-zareczynowe</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Skup diamentów Warszawa – 1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Skup diamentów Warszawa</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Skup diamentów Warszawa – uczciwa cena</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Wyceniamy brylanty i biżuterię z kamieniami. Bezpłatna wycena w salonie. Szybka płatność.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>https://forumjubiler.pl/skup-diamentow</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Wycena brylantów – 1</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Wycena brylantów</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Wycena brylantu – bezpłatna konsultacja</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Certyfikowany gemmolog wyceni Twój diament. Forum Jubiler, Chłodna 22, Warszawa.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>https://forumjubiler.pl/skup-diamentow</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Certyfikat GIA – 1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Certyfikat GIA IGI</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Ekspertyza gemmologiczna Warszawa</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Weryfikacja certyfikatu GIA/IGI, ocena kamieni, ekspertyzy biżuterii. Forum Jubiler od 1992.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>https://forumjubiler.pl/ekspertyzy</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Gemmolog Warszawa – 1</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Gemmolog Warszawa</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Gemmolog Warszawa – wycena i ekspertyzy</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Profesjonalne ekspertyzy biżuterii i kamieni szlachetnych. Umów wizytę online.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>https://forumjubiler.pl/ekspertyzy</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Forum Jubiler brand – 1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Forum Jubiler marka</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Forum Jubiler – złotnik Warszawa od 1992</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Pierścionki zaręczynowe, diamenty, ekspertyzy. Autorska biżuteria na zamówienie. Chłodna 22.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>https://forumjubiler.pl</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix OpenAI Ads XLSX validation errors
- target_countries: changed to JSON array ["PL"]
- objective: lowercase (conversions/impressions)
- ads sheet: added title, copy, link, image_link columns

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K23AdRzfbK9DAxfNeDXX3m
</commit_message>
<xml_diff>
--- a/output/openai-ads-kampanie.xlsx
+++ b/output/openai-ads-kampanie.xlsx
@@ -556,13 +556,17 @@
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>CONVERSIONS</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
+          <t>conversions</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>UZUPEŁNIJ_ID</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>["PL"]</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
@@ -593,13 +597,17 @@
       <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>CONVERSIONS</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr"/>
+          <t>conversions</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>UZUPEŁNIJ_ID</t>
+        </is>
+      </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>["PL"]</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr"/>
@@ -630,13 +638,17 @@
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>CONVERSIONS</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
+          <t>conversions</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>UZUPEŁNIJ_ID</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>["PL"]</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
@@ -667,13 +679,17 @@
       <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>CONVERSIONS</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr"/>
+          <t>conversions</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>UZUPEŁNIJ_ID</t>
+        </is>
+      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>["PL"]</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr"/>
@@ -704,13 +720,13 @@
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>AWARENESS</t>
+          <t>impressions</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>["PL"]</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
@@ -931,16 +947,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -961,30 +978,35 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>headline</t>
+          <t>title</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>copy</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>final_url</t>
+          <t>link</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>image_link</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2" ht="45" customHeight="1">
       <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Zaręczyny Warszawa – Pierścionki</t>
+          <t>Zaręczyny Warszawa 1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1009,15 +1031,20 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="40" customHeight="1">
+          <t>UZUPEŁNIJ_URL_OBRAZKA</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
       <c r="A3" s="3" t="inlineStr"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Pierścionki na zamówienie – 1</t>
+          <t>Pierścionki na zamówienie 1</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1042,15 +1069,20 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
+          <t>UZUPEŁNIJ_URL_OBRAZKA</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1">
       <c r="A4" s="2" t="inlineStr"/>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Diamenty certyfikowane – 1</t>
+          <t>Diamenty certyfikowane 1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1075,15 +1107,20 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
+          <t>UZUPEŁNIJ_URL_OBRAZKA</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
       <c r="A5" s="3" t="inlineStr"/>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Pierścionek zaręczynowy – 1</t>
+          <t>Pierścionek zaręczynowy 1</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1108,15 +1145,20 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
+          <t>UZUPEŁNIJ_URL_OBRAZKA</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="inlineStr"/>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Skup diamentów Warszawa – 1</t>
+          <t>Skup diamentów 1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1141,15 +1183,20 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
+          <t>UZUPEŁNIJ_URL_OBRAZKA</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
       <c r="A7" s="3" t="inlineStr"/>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Wycena brylantów – 1</t>
+          <t>Wycena brylantów 1</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1174,15 +1221,20 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
+          <t>UZUPEŁNIJ_URL_OBRAZKA</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="inlineStr"/>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Certyfikat GIA – 1</t>
+          <t>Certyfikat GIA 1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1207,15 +1259,20 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
+          <t>UZUPEŁNIJ_URL_OBRAZKA</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="3" t="inlineStr"/>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Gemmolog Warszawa – 1</t>
+          <t>Gemmolog Warszawa 1</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1240,15 +1297,20 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
+          <t>UZUPEŁNIJ_URL_OBRAZKA</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
       <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Forum Jubiler brand – 1</t>
+          <t>Forum Jubiler brand 1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1272,6 +1334,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>UZUPEŁNIJ_URL_OBRAZKA</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>

</xml_diff>